<commit_message>
Check in generated workbook and deliverable updates
</commit_message>
<xml_diff>
--- a/deliverables/bilal_ganj_master_market_pack_v17_20260416_032251/j40_hardware_remaining_dedup_v1_20260416.xlsx
+++ b/deliverables/bilal_ganj_master_market_pack_v17_20260416_032251/j40_hardware_remaining_dedup_v1_20260416.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -690,32 +690,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Fuse box - Compact covered ATO/ATC fuse block 6-way</t>
+          <t>Heat plugs / glow plugs - Diesel glow plug set (thread/reach/voltage per engine code)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>3 identical</t>
+          <t>Full set</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>29</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>PKR 11100-21000</t>
+          <t>PKR 12000-36000</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>11100</v>
+        <v>12000</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>21000</v>
+        <v>36000</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>16050</v>
+        <v>24000</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -736,32 +736,32 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Heat plugs / glow plugs - Diesel glow plug set (thread/reach/voltage per engine code)</t>
+          <t>Kit A nut - M10 nyloc/all-metal mix</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Full set</t>
+          <t>24 (+20% spare)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>244</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>PKR 12000-36000</t>
+          <t>PKR 1200-2400</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>12000</v>
+        <v>1200</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>36000</v>
+        <v>2400</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>24000</v>
+        <v>1800</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -782,12 +782,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Kit A nut - M10 nyloc/all-metal mix</t>
+          <t>Kit A nut - M12 nut</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>24 (+20% spare)</t>
+          <t>6 (+20% spare)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>PKR 1200-2400</t>
+          <t>PKR 500-1100</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>2400</v>
+        <v>1100</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>1800</v>
+        <v>800</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -828,12 +828,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Kit A nut - M12 nut</t>
+          <t>Kit A sleeve/spacer - Sleeve for M10 mount points</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>6 (+20% spare)</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -843,17 +843,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>PKR 500-1100</t>
+          <t>PKR 1200-3200</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>500</v>
+        <v>1200</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1100</v>
+        <v>3200</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>800</v>
+        <v>2200</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -874,12 +874,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Kit A sleeve/spacer - Sleeve for M10 mount points</t>
+          <t>Kit A spring washer - M10 spring washer</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20 (+20% spare)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -889,17 +889,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>PKR 1200-3200</t>
+          <t>PKR 300-650</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1200</v>
+        <v>300</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>3200</v>
+        <v>650</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>2200</v>
+        <v>475</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -920,12 +920,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Kit A spring washer - M10 spring washer</t>
+          <t>Kit A spring washer - M12 spring washer</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>20 (+20% spare)</t>
+          <t>6 (+20% spare)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -935,17 +935,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>PKR 300-650</t>
+          <t>PKR 150-350</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>650</v>
+        <v>350</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>475</v>
+        <v>250</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -966,12 +966,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Kit A spring washer - M12 spring washer</t>
+          <t>Kit A washer - M10 flat washer</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>6 (+20% spare)</t>
+          <t>40 (+20% spare)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -981,17 +981,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>PKR 150-350</t>
+          <t>PKR 400-900</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>350</v>
+        <v>900</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>250</v>
+        <v>650</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -1012,12 +1012,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Kit A washer - M10 flat washer</t>
+          <t>Kit A washer - M12 flat washer</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>40 (+20% spare)</t>
+          <t>12 (+20% spare)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1027,17 +1027,17 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>PKR 400-900</t>
+          <t>PKR 200-500</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>900</v>
+        <v>500</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>650</v>
+        <v>350</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1058,32 +1058,32 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Kit A washer - M12 flat washer</t>
+          <t>Kit B bolt - M6x1.0 class 8.8 hex bolts lengths 12/16/20/25mm</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>12 (+20% spare)</t>
+          <t>220 total</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>244</t>
+          <t>245</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>PKR 200-500</t>
+          <t>PKR 6000-13000</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>200</v>
+        <v>6000</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>500</v>
+        <v>13000</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>350</v>
+        <v>9500</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1104,12 +1104,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Kit B bolt - M6x1.0 class 8.8 hex bolts lengths 12/16/20/25mm</t>
+          <t>Kit B bolt - M8x1.25 class 8.8 bolts lengths 16/20/25/30mm</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>220 total</t>
+          <t>120 total</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1119,17 +1119,17 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>PKR 6000-13000</t>
+          <t>PKR 4800-10800</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>6000</v>
+        <v>4800</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>13000</v>
+        <v>10800</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>9500</v>
+        <v>7800</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1150,12 +1150,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Kit B bolt - M8x1.25 class 8.8 bolts lengths 16/20/25/30mm</t>
+          <t>Kit B nuts - M6 flange nuts</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>120 total</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1165,17 +1165,17 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>PKR 4800-10800</t>
+          <t>PKR 1200-2800</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>4800</v>
+        <v>1200</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>10800</v>
+        <v>2800</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>7800</v>
+        <v>2000</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1196,12 +1196,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kit B nuts - M6 flange nuts</t>
+          <t>Kit B nuts - M6 nyloc</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>160</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1211,17 +1211,17 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>PKR 1200-2800</t>
+          <t>PKR 3200-6400</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1200</v>
+        <v>3200</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>2800</v>
+        <v>6400</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>2000</v>
+        <v>4800</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1242,12 +1242,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kit B nuts - M6 nyloc</t>
+          <t>Kit B nuts - M8 flange nuts</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1257,17 +1257,17 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>PKR 3200-6400</t>
+          <t>PKR 1000-2200</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>3200</v>
+        <v>1000</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>6400</v>
+        <v>2200</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>4800</v>
+        <v>1600</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1288,12 +1288,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Kit B nuts - M8 flange nuts</t>
+          <t>Kit B nuts - M8 nyloc</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1303,17 +1303,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>PKR 1000-2200</t>
+          <t>PKR 2700-6300</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>1000</v>
+        <v>2700</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>2200</v>
+        <v>6300</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>1600</v>
+        <v>4500</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1334,12 +1334,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Kit B nuts - M8 nyloc</t>
+          <t>Kit B spring washers - M6 spring washers</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>140</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1349,17 +1349,17 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>PKR 2700-6300</t>
+          <t>PKR 600-1700</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>2700</v>
+        <v>600</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>6300</v>
+        <v>1700</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>4500</v>
+        <v>1150</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1380,12 +1380,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Kit B spring washers - M6 spring washers</t>
+          <t>Kit B spring washers - M8 spring washers</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1395,17 +1395,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>PKR 600-1700</t>
+          <t>PKR 600-1600</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
         <v>600</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>1700</v>
+        <v>1600</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>1150</v>
+        <v>1100</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1426,12 +1426,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Kit B spring washers - M8 spring washers</t>
+          <t>Kit B washers - M6 flat washers</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>300</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1441,17 +1441,17 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>PKR 600-1600</t>
+          <t>PKR 900-2400</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1600</v>
+        <v>2400</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>1100</v>
+        <v>1650</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1472,12 +1472,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Kit B washers - M6 flat washers</t>
+          <t>Kit B washers - M8 flat washers</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>180</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1487,17 +1487,17 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>PKR 900-2400</t>
+          <t>PKR 900-2500</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
         <v>900</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>2400</v>
+        <v>2500</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>1650</v>
+        <v>1700</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -1518,32 +1518,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Kit B washers - M8 flat washers</t>
+          <t>Kit C captive nut - M6 captive/clip nuts</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>120</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>245</t>
+          <t>246</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>PKR 900-2500</t>
+          <t>PKR 1800-4200</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>900</v>
+        <v>1800</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>2500</v>
+        <v>4200</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>1700</v>
+        <v>3000</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1564,12 +1564,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Kit C captive nut - M6 captive/clip nuts</t>
+          <t>Kit C captive nut - M8 captive/clip nuts</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1579,17 +1579,17 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>PKR 1800-4200</t>
+          <t>PKR 1500-3300</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>1800</v>
+        <v>1500</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>4200</v>
+        <v>3300</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>3000</v>
+        <v>2400</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -1610,12 +1610,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Kit C captive nut - M8 captive/clip nuts</t>
+          <t>Kit C rivnut - M6 steel rivnuts</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1625,17 +1625,17 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>PKR 1500-3300</t>
+          <t>PKR 900-2100</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
+        <v>900</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G26" s="2" t="n">
         <v>1500</v>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>3300</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>2400</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -1656,12 +1656,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Kit C rivnut - M6 steel rivnuts</t>
+          <t>Kit C rivnut - M8 steel rivnuts</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1671,17 +1671,17 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>PKR 900-2100</t>
+          <t>PKR 900-2200</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
         <v>900</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>2100</v>
+        <v>2200</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>1500</v>
+        <v>1550</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -1702,12 +1702,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Kit C rivnut - M8 steel rivnuts</t>
+          <t>Kit C weld nut - M6 weld nuts</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1717,17 +1717,17 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>PKR 900-2200</t>
+          <t>PKR 600-1500</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>2200</v>
+        <v>1500</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>1550</v>
+        <v>1050</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -1748,12 +1748,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Kit C weld nut - M6 weld nuts</t>
+          <t>Kit C weld nut - M8 weld nuts</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1763,17 +1763,17 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>PKR 600-1500</t>
+          <t>PKR 700-1600</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>1500</v>
+        <v>1600</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>1050</v>
+        <v>1150</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -1794,32 +1794,32 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Kit C weld nut - M8 weld nuts</t>
+          <t>Kit D flange nut - M6 serrated flange nut</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>247</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>PKR 700-1600</t>
+          <t>PKR 800-1800</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>1150</v>
+        <v>1300</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -1840,12 +1840,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Kit D flange nut - M6 serrated flange nut</t>
+          <t>Kit D flange nut - M8 serrated flange nut</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1855,17 +1855,17 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>PKR 800-1800</t>
+          <t>PKR 700-1500</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>1800</v>
+        <v>1500</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>1300</v>
+        <v>1100</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -1886,12 +1886,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Kit D flange nut - M8 serrated flange nut</t>
+          <t>Kit D star washer - M10 star/serrated washer</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1901,17 +1901,17 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>PKR 700-1500</t>
+          <t>PKR 700-1700</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
         <v>700</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>1500</v>
+        <v>1700</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -1932,12 +1932,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Kit D star washer - M10 star/serrated washer</t>
+          <t>Kit D star washer - M6 star/serrated washer</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>120</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1947,17 +1947,17 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>PKR 700-1700</t>
+          <t>PKR 700-1800</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
         <v>700</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1700</v>
+        <v>1800</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>1200</v>
+        <v>1250</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
@@ -1978,12 +1978,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Kit D star washer - M6 star/serrated washer</t>
+          <t>Kit D star washer - M8 star/serrated washer</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1993,17 +1993,17 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>PKR 700-1800</t>
+          <t>PKR 800-2200</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>1800</v>
+        <v>2200</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>1250</v>
+        <v>1500</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -2024,32 +2024,32 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Kit D star washer - M8 star/serrated washer</t>
+          <t>Local front leaf spring pack (new, custom to measured dimensions)</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>2 packs</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>247</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>PKR 800-2200</t>
+          <t>PKR 35000-90000</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>800</v>
+        <v>35000</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>2200</v>
+        <v>90000</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>1500</v>
+        <v>62500</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -2063,14 +2063,14 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>AS_LISTED</t>
+          <t>MEASURE_FIRST_THEN_BUY</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Local front leaf spring pack (new, custom to measured dimensions)</t>
+          <t>Local rear leaf spring pack (new, custom to measured dimensions)</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2116,32 +2116,32 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Local rear leaf spring pack (new, custom to measured dimensions)</t>
+          <t>Rear anti-inversion kit - FK08 (spring flip prevention)</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>2 packs</t>
+          <t>1 kit</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>SUS-10</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>PKR 35000-90000</t>
+          <t>PKR 12000-35000</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F37" s="2" t="n">
         <v>35000</v>
       </c>
-      <c r="F37" s="2" t="n">
-        <v>90000</v>
-      </c>
       <c r="G37" s="2" t="n">
-        <v>62500</v>
+        <v>23500</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
@@ -2155,39 +2155,39 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>MEASURE_FIRST_THEN_BUY</t>
+          <t>BUY_ONLY_IF_INVERSION_RISK</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Rear anti-inversion kit - FK08 (spring flip prevention)</t>
+          <t>Shims/spacers - M10/M12 shim pack thickness 1/2/3/5mm</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>1 kit</t>
+          <t>Assorted full pack</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>SUS-10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>PKR 12000-35000</t>
+          <t>PKR 3000-12000</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F38" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="F38" s="2" t="n">
-        <v>35000</v>
-      </c>
       <c r="G38" s="2" t="n">
-        <v>23500</v>
+        <v>7500</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -2201,39 +2201,39 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>BUY_ONLY_IF_INVERSION_RISK</t>
+          <t>AS_LISTED</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Shims/spacers - M10/M12 shim pack thickness 1/2/3/5mm</t>
+          <t>Shock absorbers (new genuine, Pakistan high-quality path)</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Assorted full pack</t>
+          <t>1 full set (front+rear)</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>SUS-11</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>PKR 3000-12000</t>
+          <t>PKR 25,000-80,000 (quote by exact model fitment)</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>3000</v>
+        <v>25000</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>12000</v>
+        <v>80000</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>7500</v>
+        <v>52500</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -2247,39 +2247,39 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>AS_LISTED</t>
+          <t>QUOTE_FIRST_THEN_BUY</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Shock absorbers (new genuine, Pakistan high-quality path)</t>
+          <t>Steering bushings - Steering linkage bush set</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>1 full set (front+rear)</t>
+          <t>1 set</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>SUS-11</t>
+          <t>230</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>PKR 25,000-80,000 (quote by exact model fitment)</t>
+          <t>PKR 3000-12000</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>25000</v>
+        <v>3000</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>80000</v>
+        <v>12000</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>52500</v>
+        <v>7500</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -2293,80 +2293,34 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>QUOTE_FIRST_THEN_BUY</t>
+          <t>BUY_ONLY_IF_PLAY_FOUND</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Steering bushings - Steering linkage bush set</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>1 set</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>230</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>PKR 3000-12000</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F41" s="2" t="n">
-        <v>12000</v>
-      </c>
-      <c r="G41" s="2" t="n">
-        <v>7500</v>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>NOT_PURCHASED</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>BUY_ONLY_IF_PLAY_FOUND</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B42" s="3" t="n"/>
-      <c r="C42" s="3" t="n"/>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3">
+      <c r="B41" s="3" t="n"/>
+      <c r="C41" s="3" t="n"/>
+      <c r="D41" s="3" t="n"/>
+      <c r="E41" s="3">
         <f>SUM(E2:E41)</f>
         <v/>
       </c>
-      <c r="F42" s="3">
+      <c r="F41" s="3">
         <f>SUM(F2:F41)</f>
         <v/>
       </c>
-      <c r="G42" s="3">
+      <c r="G41" s="3">
         <f>SUM(G2:G41)</f>
         <v/>
       </c>
-      <c r="H42" s="3" t="n"/>
-      <c r="I42" s="3" t="n"/>
-      <c r="J42" s="3" t="n"/>
+      <c r="H41" s="3" t="n"/>
+      <c r="I41" s="3" t="n"/>
+      <c r="J41" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J42"/>

</xml_diff>